<commit_message>
perf: write back loaded shared formulas on save (#692)
A save now writes each shared formula a load brought in back as a shared
formula, limited to the cells that still hold it (XLCellFormula.TryGetShared:
text and position unchanged since the load). Nothing is parsed at save.
Edits, moves, shifts, copies and rename rewrites drop a cell from its group.
New groups are never searched for, as Excel itself never does.

The rules come from ECMA-376 and from Excel over COM: master first in the
sheet and top-left of ref, every follower inside ref, si dense from 0 per
sheet, no sheet or structured references, no #REF! cells.

ADR 0003 records the decision and the measurements.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/Cubes/CubeFromRange-Output.xlsx
+++ b/XLibur.Tests/Resource/Other/Cubes/CubeFromRange-Output.xlsx
@@ -701,11 +701,11 @@
         <x:v>Baclava</x:v>
       </x:c>
       <x:c r="B4" vm="13">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A4,B$3)</x:f>
+        <x:f t="shared" ref="B4:C7" si="0">CUBEVALUE("ThisWorkbookDataModel",$A4,B$3)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="C4" vm="14">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A4,C$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -715,11 +715,11 @@
         <x:v>Cake</x:v>
       </x:c>
       <x:c r="B5" vm="11">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A5,B$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C5" vm="12">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A5,C$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>27</x:v>
       </x:c>
     </x:row>
@@ -729,11 +729,11 @@
         <x:v>Pie</x:v>
       </x:c>
       <x:c r="B6" vm="9">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A6,B$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>12</x:v>
       </x:c>
       <x:c r="C6" vm="10">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A6,C$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>35</x:v>
       </x:c>
     </x:row>
@@ -743,11 +743,11 @@
         <x:v>Grand Total</x:v>
       </x:c>
       <x:c r="B7" vm="7">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A7,B$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>33</x:v>
       </x:c>
       <x:c r="C7" vm="8">
-        <x:f>CUBEVALUE("ThisWorkbookDataModel",$A7,C$3)</x:f>
+        <x:f t="shared" si="0"/>
         <x:v>65</x:v>
       </x:c>
     </x:row>

</xml_diff>